<commit_message>
new agent for capacity added
</commit_message>
<xml_diff>
--- a/Jobsdata.xlsx
+++ b/Jobsdata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="47">
   <si>
     <t>POSTING_DATE</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>2026-06-02</t>
+  </si>
+  <si>
+    <t>2026-06-03</t>
   </si>
   <si>
     <t>İSTANBUL</t>
@@ -509,7 +512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -549,16 +552,16 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2">
         <v>7381125</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F2">
         <v>19</v>
@@ -581,16 +584,16 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3">
         <v>2207663</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3">
         <v>15</v>
@@ -613,16 +616,16 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>7397528</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4">
         <v>29</v>
@@ -645,16 +648,16 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5">
         <v>5931712</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F5">
         <v>15</v>
@@ -677,16 +680,16 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>7325488</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F6">
         <v>10</v>
@@ -709,16 +712,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>3368175</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7">
         <v>20</v>
@@ -741,16 +744,16 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8">
         <v>3864716</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F8">
         <v>21</v>
@@ -773,16 +776,16 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9">
         <v>3367403</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -805,16 +808,16 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D10">
         <v>7381124</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F10">
         <v>29</v>
@@ -837,16 +840,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D11">
         <v>7079978</v>
       </c>
       <c r="E11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F11">
         <v>6</v>
@@ -869,16 +872,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D12">
         <v>3367739</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F12">
         <v>3</v>
@@ -901,16 +904,16 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13">
         <v>7072286</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -933,16 +936,16 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D14">
         <v>3367743</v>
       </c>
       <c r="E14" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -965,16 +968,16 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15">
         <v>4214024</v>
       </c>
       <c r="E15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -997,16 +1000,16 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16">
         <v>7357843</v>
       </c>
       <c r="E16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F16">
         <v>16</v>
@@ -1029,16 +1032,16 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D17">
         <v>7077448</v>
       </c>
       <c r="E17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -1061,16 +1064,16 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D18">
         <v>2278099</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F18">
         <v>20</v>
@@ -1093,16 +1096,16 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C19" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D19">
         <v>7077738</v>
       </c>
       <c r="E19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F19">
         <v>2</v>
@@ -1125,16 +1128,16 @@
         <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D20">
         <v>4493936</v>
       </c>
       <c r="E20" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F20">
         <v>8</v>
@@ -1157,16 +1160,16 @@
         <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D21">
         <v>5284531</v>
       </c>
       <c r="E21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F21">
         <v>4</v>
@@ -1189,16 +1192,16 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C22" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D22">
         <v>5954007</v>
       </c>
       <c r="E22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F22">
         <v>26</v>
@@ -1221,16 +1224,16 @@
         <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C23" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D23">
         <v>7081903</v>
       </c>
       <c r="E23" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F23">
         <v>11</v>
@@ -1253,16 +1256,16 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C24" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D24">
         <v>9366541</v>
       </c>
       <c r="E24" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F24">
         <v>25</v>
@@ -1285,16 +1288,16 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D25">
         <v>6435172</v>
       </c>
       <c r="E25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1317,16 +1320,16 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C26" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D26">
         <v>7077736</v>
       </c>
       <c r="E26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -1349,16 +1352,16 @@
         <v>11</v>
       </c>
       <c r="B27" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D27">
         <v>7381125</v>
       </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F27">
         <v>24</v>
@@ -1381,16 +1384,16 @@
         <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D28">
         <v>2207663</v>
       </c>
       <c r="E28" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F28">
         <v>16</v>
@@ -1413,16 +1416,16 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D29">
         <v>7397528</v>
       </c>
       <c r="E29" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F29">
         <v>32</v>
@@ -1445,16 +1448,16 @@
         <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D30">
         <v>5931712</v>
       </c>
       <c r="E30" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F30">
         <v>13</v>
@@ -1477,16 +1480,16 @@
         <v>11</v>
       </c>
       <c r="B31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D31">
         <v>7325488</v>
       </c>
       <c r="E31" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F31">
         <v>18</v>
@@ -1509,16 +1512,16 @@
         <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D32">
         <v>3368175</v>
       </c>
       <c r="E32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F32">
         <v>22</v>
@@ -1541,16 +1544,16 @@
         <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D33">
         <v>3864716</v>
       </c>
       <c r="E33" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F33">
         <v>30</v>
@@ -1573,16 +1576,16 @@
         <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D34">
         <v>3367403</v>
       </c>
       <c r="E34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F34">
         <v>4</v>
@@ -1605,16 +1608,16 @@
         <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D35">
         <v>7381124</v>
       </c>
       <c r="E35" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F35">
         <v>36</v>
@@ -1637,16 +1640,16 @@
         <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C36" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D36">
         <v>7079978</v>
       </c>
       <c r="E36" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F36">
         <v>4</v>
@@ -1669,16 +1672,16 @@
         <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C37" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D37">
         <v>3367739</v>
       </c>
       <c r="E37" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F37">
         <v>4</v>
@@ -1701,16 +1704,16 @@
         <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C38" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D38">
         <v>7072286</v>
       </c>
       <c r="E38" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F38">
         <v>3</v>
@@ -1733,16 +1736,16 @@
         <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C39" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D39">
         <v>3367743</v>
       </c>
       <c r="E39" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -1765,16 +1768,16 @@
         <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C40" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D40">
         <v>4214024</v>
       </c>
       <c r="E40" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -1797,16 +1800,16 @@
         <v>11</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C41" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D41">
         <v>7357843</v>
       </c>
       <c r="E41" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F41">
         <v>16</v>
@@ -1829,16 +1832,16 @@
         <v>11</v>
       </c>
       <c r="B42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D42">
         <v>7077448</v>
       </c>
       <c r="E42" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F42">
         <v>1</v>
@@ -1861,16 +1864,16 @@
         <v>11</v>
       </c>
       <c r="B43" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C43" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D43">
         <v>2278099</v>
       </c>
       <c r="E43" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F43">
         <v>28</v>
@@ -1893,16 +1896,16 @@
         <v>11</v>
       </c>
       <c r="B44" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C44" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D44">
         <v>7077738</v>
       </c>
       <c r="E44" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F44">
         <v>4</v>
@@ -1925,16 +1928,16 @@
         <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C45" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D45">
         <v>4493936</v>
       </c>
       <c r="E45" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F45">
         <v>10</v>
@@ -1957,16 +1960,16 @@
         <v>11</v>
       </c>
       <c r="B46" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C46" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D46">
         <v>5284531</v>
       </c>
       <c r="E46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F46">
         <v>3</v>
@@ -1989,16 +1992,16 @@
         <v>11</v>
       </c>
       <c r="B47" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C47" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D47">
         <v>5954007</v>
       </c>
       <c r="E47" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F47">
         <v>23</v>
@@ -2021,16 +2024,16 @@
         <v>11</v>
       </c>
       <c r="B48" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C48" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D48">
         <v>7081903</v>
       </c>
       <c r="E48" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F48">
         <v>10</v>
@@ -2053,16 +2056,16 @@
         <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C49" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D49">
         <v>9366541</v>
       </c>
       <c r="E49" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F49">
         <v>27</v>
@@ -2085,16 +2088,16 @@
         <v>11</v>
       </c>
       <c r="B50" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C50" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D50">
         <v>6435172</v>
       </c>
       <c r="E50" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F50">
         <v>2</v>
@@ -2117,16 +2120,16 @@
         <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C51" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D51">
         <v>7077736</v>
       </c>
       <c r="E51" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F51">
         <v>0</v>
@@ -2142,6 +2145,806 @@
       </c>
       <c r="J51">
         <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10">
+      <c r="A52" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" t="s">
+        <v>13</v>
+      </c>
+      <c r="C52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52">
+        <v>7381125</v>
+      </c>
+      <c r="E52" t="s">
+        <v>22</v>
+      </c>
+      <c r="F52">
+        <v>27</v>
+      </c>
+      <c r="G52">
+        <v>25</v>
+      </c>
+      <c r="H52">
+        <v>5</v>
+      </c>
+      <c r="I52">
+        <v>7</v>
+      </c>
+      <c r="J52">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
+      <c r="A53" t="s">
+        <v>12</v>
+      </c>
+      <c r="B53" t="s">
+        <v>13</v>
+      </c>
+      <c r="C53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53">
+        <v>2207663</v>
+      </c>
+      <c r="E53" t="s">
+        <v>23</v>
+      </c>
+      <c r="F53">
+        <v>19</v>
+      </c>
+      <c r="G53">
+        <v>15</v>
+      </c>
+      <c r="H53">
+        <v>2</v>
+      </c>
+      <c r="I53">
+        <v>6</v>
+      </c>
+      <c r="J53">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10">
+      <c r="A54" t="s">
+        <v>12</v>
+      </c>
+      <c r="B54" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54">
+        <v>7397528</v>
+      </c>
+      <c r="E54" t="s">
+        <v>24</v>
+      </c>
+      <c r="F54">
+        <v>28</v>
+      </c>
+      <c r="G54">
+        <v>22</v>
+      </c>
+      <c r="H54">
+        <v>6</v>
+      </c>
+      <c r="I54">
+        <v>25</v>
+      </c>
+      <c r="J54">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
+      <c r="A55" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" t="s">
+        <v>13</v>
+      </c>
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55">
+        <v>5931712</v>
+      </c>
+      <c r="E55" t="s">
+        <v>25</v>
+      </c>
+      <c r="F55">
+        <v>13</v>
+      </c>
+      <c r="G55">
+        <v>15</v>
+      </c>
+      <c r="H55">
+        <v>4</v>
+      </c>
+      <c r="I55">
+        <v>16</v>
+      </c>
+      <c r="J55">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
+      <c r="A56" t="s">
+        <v>12</v>
+      </c>
+      <c r="B56" t="s">
+        <v>13</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56">
+        <v>7325488</v>
+      </c>
+      <c r="E56" t="s">
+        <v>26</v>
+      </c>
+      <c r="F56">
+        <v>28</v>
+      </c>
+      <c r="G56">
+        <v>40</v>
+      </c>
+      <c r="H56">
+        <v>8</v>
+      </c>
+      <c r="I56">
+        <v>15</v>
+      </c>
+      <c r="J56">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10">
+      <c r="A57" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" t="s">
+        <v>13</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>3368175</v>
+      </c>
+      <c r="E57" t="s">
+        <v>27</v>
+      </c>
+      <c r="F57">
+        <v>29</v>
+      </c>
+      <c r="G57">
+        <v>23</v>
+      </c>
+      <c r="H57">
+        <v>5</v>
+      </c>
+      <c r="I57">
+        <v>13</v>
+      </c>
+      <c r="J57">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10">
+      <c r="A58" t="s">
+        <v>12</v>
+      </c>
+      <c r="B58" t="s">
+        <v>13</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>3864716</v>
+      </c>
+      <c r="E58" t="s">
+        <v>28</v>
+      </c>
+      <c r="F58">
+        <v>41</v>
+      </c>
+      <c r="G58">
+        <v>19</v>
+      </c>
+      <c r="H58">
+        <v>6</v>
+      </c>
+      <c r="I58">
+        <v>9</v>
+      </c>
+      <c r="J58">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
+      <c r="A59" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C59" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59">
+        <v>3367403</v>
+      </c>
+      <c r="E59" t="s">
+        <v>29</v>
+      </c>
+      <c r="F59">
+        <v>6</v>
+      </c>
+      <c r="G59">
+        <v>9</v>
+      </c>
+      <c r="H59">
+        <v>6</v>
+      </c>
+      <c r="I59">
+        <v>8</v>
+      </c>
+      <c r="J59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
+      <c r="A60" t="s">
+        <v>12</v>
+      </c>
+      <c r="B60" t="s">
+        <v>13</v>
+      </c>
+      <c r="C60" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60">
+        <v>7381124</v>
+      </c>
+      <c r="E60" t="s">
+        <v>30</v>
+      </c>
+      <c r="F60">
+        <v>34</v>
+      </c>
+      <c r="G60">
+        <v>28</v>
+      </c>
+      <c r="H60">
+        <v>7</v>
+      </c>
+      <c r="I60">
+        <v>11</v>
+      </c>
+      <c r="J60">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
+      <c r="A61" t="s">
+        <v>12</v>
+      </c>
+      <c r="B61" t="s">
+        <v>13</v>
+      </c>
+      <c r="C61" t="s">
+        <v>14</v>
+      </c>
+      <c r="D61">
+        <v>7079978</v>
+      </c>
+      <c r="E61" t="s">
+        <v>31</v>
+      </c>
+      <c r="F61">
+        <v>7</v>
+      </c>
+      <c r="G61">
+        <v>3</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61">
+        <v>6</v>
+      </c>
+      <c r="J61">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
+      <c r="A62" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" t="s">
+        <v>14</v>
+      </c>
+      <c r="D62">
+        <v>3367739</v>
+      </c>
+      <c r="E62" t="s">
+        <v>32</v>
+      </c>
+      <c r="F62">
+        <v>4</v>
+      </c>
+      <c r="G62">
+        <v>3</v>
+      </c>
+      <c r="H62">
+        <v>1</v>
+      </c>
+      <c r="I62">
+        <v>7</v>
+      </c>
+      <c r="J62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
+      <c r="A63" t="s">
+        <v>12</v>
+      </c>
+      <c r="B63" t="s">
+        <v>13</v>
+      </c>
+      <c r="C63" t="s">
+        <v>15</v>
+      </c>
+      <c r="D63">
+        <v>7072286</v>
+      </c>
+      <c r="E63" t="s">
+        <v>33</v>
+      </c>
+      <c r="F63">
+        <v>3</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <v>2</v>
+      </c>
+      <c r="J63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
+      <c r="A64" t="s">
+        <v>12</v>
+      </c>
+      <c r="B64" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" t="s">
+        <v>16</v>
+      </c>
+      <c r="D64">
+        <v>3367743</v>
+      </c>
+      <c r="E64" t="s">
+        <v>34</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>2</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>0</v>
+      </c>
+      <c r="J64">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10">
+      <c r="A65" t="s">
+        <v>12</v>
+      </c>
+      <c r="B65" t="s">
+        <v>13</v>
+      </c>
+      <c r="C65" t="s">
+        <v>15</v>
+      </c>
+      <c r="D65">
+        <v>4214024</v>
+      </c>
+      <c r="E65" t="s">
+        <v>35</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+      <c r="G65">
+        <v>4</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>0</v>
+      </c>
+      <c r="J65">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10">
+      <c r="A66" t="s">
+        <v>12</v>
+      </c>
+      <c r="B66" t="s">
+        <v>13</v>
+      </c>
+      <c r="C66" t="s">
+        <v>16</v>
+      </c>
+      <c r="D66">
+        <v>7357843</v>
+      </c>
+      <c r="E66" t="s">
+        <v>36</v>
+      </c>
+      <c r="F66">
+        <v>17</v>
+      </c>
+      <c r="G66">
+        <v>2</v>
+      </c>
+      <c r="H66">
+        <v>2</v>
+      </c>
+      <c r="I66">
+        <v>4</v>
+      </c>
+      <c r="J66">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10">
+      <c r="A67" t="s">
+        <v>12</v>
+      </c>
+      <c r="B67" t="s">
+        <v>13</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>7077448</v>
+      </c>
+      <c r="E67" t="s">
+        <v>37</v>
+      </c>
+      <c r="F67">
+        <v>2</v>
+      </c>
+      <c r="G67">
+        <v>1</v>
+      </c>
+      <c r="H67">
+        <v>1</v>
+      </c>
+      <c r="I67">
+        <v>1</v>
+      </c>
+      <c r="J67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10">
+      <c r="A68" t="s">
+        <v>12</v>
+      </c>
+      <c r="B68" t="s">
+        <v>13</v>
+      </c>
+      <c r="C68" t="s">
+        <v>17</v>
+      </c>
+      <c r="D68">
+        <v>2278099</v>
+      </c>
+      <c r="E68" t="s">
+        <v>38</v>
+      </c>
+      <c r="F68">
+        <v>27</v>
+      </c>
+      <c r="G68">
+        <v>17</v>
+      </c>
+      <c r="H68">
+        <v>3</v>
+      </c>
+      <c r="I68">
+        <v>35</v>
+      </c>
+      <c r="J68">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10">
+      <c r="A69" t="s">
+        <v>12</v>
+      </c>
+      <c r="B69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C69" t="s">
+        <v>17</v>
+      </c>
+      <c r="D69">
+        <v>7077738</v>
+      </c>
+      <c r="E69" t="s">
+        <v>39</v>
+      </c>
+      <c r="F69">
+        <v>4</v>
+      </c>
+      <c r="G69">
+        <v>3</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>3</v>
+      </c>
+      <c r="J69">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10">
+      <c r="A70" t="s">
+        <v>12</v>
+      </c>
+      <c r="B70" t="s">
+        <v>13</v>
+      </c>
+      <c r="C70" t="s">
+        <v>17</v>
+      </c>
+      <c r="D70">
+        <v>4493936</v>
+      </c>
+      <c r="E70" t="s">
+        <v>40</v>
+      </c>
+      <c r="F70">
+        <v>7</v>
+      </c>
+      <c r="G70">
+        <v>4</v>
+      </c>
+      <c r="H70">
+        <v>1</v>
+      </c>
+      <c r="I70">
+        <v>7</v>
+      </c>
+      <c r="J70">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10">
+      <c r="A71" t="s">
+        <v>12</v>
+      </c>
+      <c r="B71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C71" t="s">
+        <v>17</v>
+      </c>
+      <c r="D71">
+        <v>5284531</v>
+      </c>
+      <c r="E71" t="s">
+        <v>41</v>
+      </c>
+      <c r="F71">
+        <v>6</v>
+      </c>
+      <c r="G71">
+        <v>3</v>
+      </c>
+      <c r="H71">
+        <v>0</v>
+      </c>
+      <c r="I71">
+        <v>1</v>
+      </c>
+      <c r="J71">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10">
+      <c r="A72" t="s">
+        <v>12</v>
+      </c>
+      <c r="B72" t="s">
+        <v>13</v>
+      </c>
+      <c r="C72" t="s">
+        <v>18</v>
+      </c>
+      <c r="D72">
+        <v>5954007</v>
+      </c>
+      <c r="E72" t="s">
+        <v>42</v>
+      </c>
+      <c r="F72">
+        <v>20</v>
+      </c>
+      <c r="G72">
+        <v>27</v>
+      </c>
+      <c r="H72">
+        <v>4</v>
+      </c>
+      <c r="I72">
+        <v>10</v>
+      </c>
+      <c r="J72">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10">
+      <c r="A73" t="s">
+        <v>12</v>
+      </c>
+      <c r="B73" t="s">
+        <v>13</v>
+      </c>
+      <c r="C73" t="s">
+        <v>18</v>
+      </c>
+      <c r="D73">
+        <v>7081903</v>
+      </c>
+      <c r="E73" t="s">
+        <v>43</v>
+      </c>
+      <c r="F73">
+        <v>14</v>
+      </c>
+      <c r="G73">
+        <v>20</v>
+      </c>
+      <c r="H73">
+        <v>2</v>
+      </c>
+      <c r="I73">
+        <v>5</v>
+      </c>
+      <c r="J73">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10">
+      <c r="A74" t="s">
+        <v>12</v>
+      </c>
+      <c r="B74" t="s">
+        <v>13</v>
+      </c>
+      <c r="C74" t="s">
+        <v>19</v>
+      </c>
+      <c r="D74">
+        <v>9366541</v>
+      </c>
+      <c r="E74" t="s">
+        <v>44</v>
+      </c>
+      <c r="F74">
+        <v>29</v>
+      </c>
+      <c r="G74">
+        <v>10</v>
+      </c>
+      <c r="H74">
+        <v>2</v>
+      </c>
+      <c r="I74">
+        <v>10</v>
+      </c>
+      <c r="J74">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10">
+      <c r="A75" t="s">
+        <v>12</v>
+      </c>
+      <c r="B75" t="s">
+        <v>13</v>
+      </c>
+      <c r="C75" t="s">
+        <v>20</v>
+      </c>
+      <c r="D75">
+        <v>6435172</v>
+      </c>
+      <c r="E75" t="s">
+        <v>45</v>
+      </c>
+      <c r="F75">
+        <v>1</v>
+      </c>
+      <c r="G75">
+        <v>5</v>
+      </c>
+      <c r="H75">
+        <v>0</v>
+      </c>
+      <c r="I75">
+        <v>3</v>
+      </c>
+      <c r="J75">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10">
+      <c r="A76" t="s">
+        <v>12</v>
+      </c>
+      <c r="B76" t="s">
+        <v>13</v>
+      </c>
+      <c r="C76" t="s">
+        <v>21</v>
+      </c>
+      <c r="D76">
+        <v>7077736</v>
+      </c>
+      <c r="E76" t="s">
+        <v>46</v>
+      </c>
+      <c r="F76">
+        <v>2</v>
+      </c>
+      <c r="G76">
+        <v>0</v>
+      </c>
+      <c r="H76">
+        <v>0</v>
+      </c>
+      <c r="I76">
+        <v>1</v>
+      </c>
+      <c r="J76">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>